<commit_message>
Final report generated and minor fixes and new plots added to the other files
</commit_message>
<xml_diff>
--- a/part1_data_collection/job-postings.xlsx
+++ b/part1_data_collection/job-postings.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs by Location" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs by Technology" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jobs by Technology1" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -528,11 +529,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C</t>
+          <t xml:space="preserve">C </t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5751</v>
+        <v>1266</v>
       </c>
     </row>
     <row r="3">
@@ -542,7 +543,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>526</v>
       </c>
     </row>
     <row r="4">
@@ -552,17 +553,17 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>506</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t xml:space="preserve">Java </t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6">
@@ -572,7 +573,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0</v>
+        <v>2248</v>
       </c>
     </row>
     <row r="7">
@@ -582,7 +583,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="8">
@@ -592,7 +593,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>138</v>
       </c>
     </row>
     <row r="9">
@@ -602,7 +603,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>899</v>
       </c>
     </row>
     <row r="10">
@@ -612,7 +613,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0</v>
+        <v>423</v>
       </c>
     </row>
     <row r="11">
@@ -632,7 +633,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>0</v>
+        <v>86</v>
       </c>
     </row>
     <row r="13">
@@ -642,7 +643,153 @@
         </is>
       </c>
       <c r="B13" t="n">
+        <v>208</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Number of Jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C </t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>1266</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>C#</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>C++</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Java</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3428</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>JavaScript</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2248</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Python</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>1173</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Scala</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Oracle</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SQL Server</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>423</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>MySQL Server</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>PostgreSQL</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MongoDB</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>